<commit_message>
fix mau hp & talic colector npc
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/19_UnitKeyItem/UnitFrame.xlsx
+++ b/gu_in/Item.edf/19_UnitKeyItem/UnitFrame.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1B1BE8-17C6-4192-A0D0-307A7F6589AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729FD935-694B-407C-8F73-F52CB4EFD5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UnitKeyItem" sheetId="1" r:id="rId1"/>
@@ -421,9 +421,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -461,9 +461,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -496,9 +496,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -531,9 +548,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -708,25 +742,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -770,7 +804,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -811,7 +845,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -853,7 +887,7 @@
         <v>tinbbb01</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -895,7 +929,7 @@
         <v>tinbbb02</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -937,7 +971,7 @@
         <v>tinbbb03</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -988,32 +1022,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AA6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1096,7 +1130,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1176,7 +1210,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -1184,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3">
-        <v>900000</v>
+        <v>300000</v>
       </c>
       <c r="D3">
         <v>0.5</v>
@@ -1256,7 +1290,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -1264,7 +1298,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="3">
-        <v>500000</v>
+        <v>150000</v>
       </c>
       <c r="D4">
         <v>0.57499998807907104</v>
@@ -1336,7 +1370,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>62</v>
       </c>
@@ -1416,7 +1450,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -1505,45 +1539,45 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AQ6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="32" max="39" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="39" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>79</v>
       </c>
@@ -1674,7 +1708,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>UnitKeyItem!A2</f>
         <v>Code</v>
@@ -1836,7 +1870,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>UnitKeyItem!A3</f>
         <v>inbbb01</v>
@@ -1948,7 +1982,7 @@
       </c>
       <c r="AD3">
         <f>UnitFrame!C3</f>
-        <v>900000</v>
+        <v>300000</v>
       </c>
       <c r="AE3">
         <f>UnitFrame!P3</f>
@@ -1998,7 +2032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>UnitKeyItem!A4</f>
         <v>inbbb02</v>
@@ -2110,7 +2144,7 @@
       </c>
       <c r="AD4">
         <f>UnitFrame!C4</f>
-        <v>500000</v>
+        <v>150000</v>
       </c>
       <c r="AE4">
         <f>UnitFrame!P4</f>
@@ -2160,7 +2194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>UnitKeyItem!A5</f>
         <v>inbbb03</v>
@@ -2322,7 +2356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>UnitKeyItem!A6</f>
         <v>inbbb04</v>
@@ -2492,9 +2526,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -2505,7 +2539,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>76</v>
       </c>
@@ -2514,7 +2548,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>0</v>
       </c>
@@ -2523,7 +2557,7 @@
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -2532,7 +2566,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>2</v>
       </c>
@@ -2541,7 +2575,7 @@
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>3</v>
       </c>

</xml_diff>